<commit_message>
Nightly lead extraction 2026-08-05
</commit_message>
<xml_diff>
--- a/UT/uta/2026-08-05.xlsx
+++ b/UT/uta/2026-08-05.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -543,7 +543,9 @@
           <t>UT</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
+      <c r="G3" t="n">
+        <v>84653</v>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>initial J matches deceased's own name 'Jarl'</t>
@@ -633,7 +635,9 @@
           <t>UT</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
+      <c r="G5" t="n">
+        <v>84003</v>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>initial B matches deceased's own name 'Batchelor'</t>
@@ -677,7 +681,9 @@
           <t>UT</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
+      <c r="G6" t="n">
+        <v>84604</v>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>initial P matches deceased's own name 'Perez'</t>
@@ -687,86 +693,6 @@
       <c r="J6" t="inlineStr">
         <is>
           <t>$475,700</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Norman B. Wall</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>WALL, NORMAN B</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>32:016:0017</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>UT</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>initial B matches deceased's own name 'B.'</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>No address on file</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>David Lee Rasmussen</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>RASMUSSEN, DAVID L</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>40:394:0002</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>173 N 800 WEST</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>SPRINGVILLE</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>UT</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>initial L matches deceased's own name 'Lee'</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>$603,400</t>
         </is>
       </c>
     </row>

</xml_diff>